<commit_message>
docs: update API endpoint descriptions and add missing feature references
</commit_message>
<xml_diff>
--- a/docs/excel/CMAS-API-Endpoints.xlsx
+++ b/docs/excel/CMAS-API-Endpoints.xlsx
@@ -1880,7 +1880,7 @@
       </c>
       <c r="I15" s="17" t="inlineStr">
         <is>
-          <t>UC 1.6</t>
+          <t>FR-22b, UC 1.6</t>
         </is>
       </c>
       <c r="J15" s="10" t="inlineStr">
@@ -2004,7 +2004,7 @@
       </c>
       <c r="I17" s="17" t="inlineStr">
         <is>
-          <t>FR-20, FR-21, FR-27, FR-28</t>
+          <t>FR-20, FR-21, FR-22c, FR-27, FR-28</t>
         </is>
       </c>
       <c r="J17" s="9" t="inlineStr">
@@ -2604,7 +2604,7 @@
       </c>
       <c r="E27" s="17" t="inlineStr">
         <is>
-          <t>เพิ่ม CLO</t>
+          <t>เพิ่ม CLO ต้องเลือกระดับ Bloom เอง ไม่มีค่าตั้งต้น</t>
         </is>
       </c>
       <c r="F27" s="17" t="inlineStr">
@@ -2624,7 +2624,7 @@
       </c>
       <c r="I27" s="17" t="inlineStr">
         <is>
-          <t>FR-30, FR-31</t>
+          <t>FR-30, FR-31, FR-99, FR-100</t>
         </is>
       </c>
       <c r="J27" s="9" t="inlineStr">
@@ -2748,7 +2748,7 @@
       </c>
       <c r="I29" s="17" t="inlineStr">
         <is>
-          <t>FR-30</t>
+          <t>FR-30, FR-99, FR-100</t>
         </is>
       </c>
       <c r="J29" s="9" t="inlineStr">
@@ -3410,7 +3410,7 @@
       </c>
       <c r="E40" s="8" t="inlineStr">
         <is>
-          <t>เมทริกซ์ กิจกรรม × จุดประสงค์</t>
+          <t>เมทริกซ์ กิจกรรม × จุดประสงค์ พร้อมคำเตือน</t>
         </is>
       </c>
       <c r="F40" s="8" t="inlineStr">
@@ -3430,7 +3430,7 @@
       </c>
       <c r="I40" s="8" t="inlineStr">
         <is>
-          <t>FR-44, FR-45, FR-48</t>
+          <t>FR-44, FR-45, FR-48, FR-102</t>
         </is>
       </c>
       <c r="J40" s="9" t="inlineStr">

</xml_diff>